<commit_message>
Added VLOOKUP and XLOOKUP practice
</commit_message>
<xml_diff>
--- a/excel.xlsx
+++ b/excel.xlsx
@@ -8,21 +8,34 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\ANALYTICS_ALL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C2F26AD4-4B8F-4714-B00A-3EB8393AC96D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1BA2525-1394-45A9-BAEC-2041062E85BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{8F9F4605-7EB3-4A88-B33F-B5AAE575BD10}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{8F9F4605-7EB3-4A88-B33F-B5AAE575BD10}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="4" r:id="rId3"/>
+    <sheet name="xlookup and vlookup" sheetId="6" r:id="rId4"/>
+    <sheet name="Sheet6" sheetId="7" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="195">
   <si>
     <t>Order ID</t>
   </si>
@@ -520,6 +533,93 @@
   </si>
   <si>
     <t>Office Supplies.Bengaluru@gmail.com</t>
+  </si>
+  <si>
+    <t>Employee ID</t>
+  </si>
+  <si>
+    <t>Employee Name</t>
+  </si>
+  <si>
+    <t>Department</t>
+  </si>
+  <si>
+    <t>Salary</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>E101</t>
+  </si>
+  <si>
+    <t>Rahul</t>
+  </si>
+  <si>
+    <t>Bangalore</t>
+  </si>
+  <si>
+    <t>E102</t>
+  </si>
+  <si>
+    <t>Priya</t>
+  </si>
+  <si>
+    <t>HR</t>
+  </si>
+  <si>
+    <t>E103</t>
+  </si>
+  <si>
+    <t>Arjun</t>
+  </si>
+  <si>
+    <t>Finance</t>
+  </si>
+  <si>
+    <t>E104</t>
+  </si>
+  <si>
+    <t>Sneha</t>
+  </si>
+  <si>
+    <t>E105</t>
+  </si>
+  <si>
+    <t>Kiran</t>
+  </si>
+  <si>
+    <t>E106</t>
+  </si>
+  <si>
+    <t>Ananya</t>
+  </si>
+  <si>
+    <t>E107</t>
+  </si>
+  <si>
+    <t>Rohit</t>
+  </si>
+  <si>
+    <t>E108</t>
+  </si>
+  <si>
+    <t>Meera</t>
+  </si>
+  <si>
+    <t>E109</t>
+  </si>
+  <si>
+    <t>Vikram</t>
+  </si>
+  <si>
+    <t>E110</t>
+  </si>
+  <si>
+    <t>Divya</t>
+  </si>
+  <si>
+    <t>Search Employee ID</t>
   </si>
 </sst>
 </file>
@@ -1009,9 +1109,21 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -4066,4 +4178,435 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B65A835-8955-4036-A2B9-F197560A1102}">
+  <dimension ref="A1:Q11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="8" max="8" width="11.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="G1" t="s">
+        <v>194</v>
+      </c>
+      <c r="H1" t="s">
+        <v>167</v>
+      </c>
+      <c r="I1" t="s">
+        <v>168</v>
+      </c>
+      <c r="J1" t="s">
+        <v>169</v>
+      </c>
+      <c r="K1" t="s">
+        <v>170</v>
+      </c>
+      <c r="M1" t="s">
+        <v>194</v>
+      </c>
+      <c r="N1" t="s">
+        <v>167</v>
+      </c>
+      <c r="O1" t="s">
+        <v>168</v>
+      </c>
+      <c r="P1" t="s">
+        <v>169</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D2" s="3">
+        <v>45000</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="G2" t="s">
+        <v>177</v>
+      </c>
+      <c r="H2" t="str">
+        <f>VLOOKUP(G2,A2:E11,2,FALSE)</f>
+        <v>Arjun</v>
+      </c>
+      <c r="I2" t="str">
+        <f>VLOOKUP(G2,A2:E11,3,FALSE)</f>
+        <v>Finance</v>
+      </c>
+      <c r="J2">
+        <f>VLOOKUP(G2,A2:E11,4,FALSE)</f>
+        <v>52000</v>
+      </c>
+      <c r="K2" t="str">
+        <f>VLOOKUP(G2,A2:E11,5,FALSE)</f>
+        <v>Chennai</v>
+      </c>
+      <c r="M2" t="s">
+        <v>174</v>
+      </c>
+      <c r="N2" t="str">
+        <f>_xlfn.XLOOKUP(M2,A2:A11,B2:B11)</f>
+        <v>Priya</v>
+      </c>
+      <c r="O2" t="str">
+        <f>_xlfn.XLOOKUP(M2,A2:A11,C2:C11)</f>
+        <v>HR</v>
+      </c>
+      <c r="P2">
+        <f>_xlfn.XLOOKUP(M2,A2:A11,D2:D11)</f>
+        <v>42000</v>
+      </c>
+      <c r="Q2" t="str">
+        <f>_xlfn.XLOOKUP(M2,A2:A11,E2:E11)</f>
+        <v>Mumbai</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="D3" s="3">
+        <v>42000</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" t="s">
+        <v>186</v>
+      </c>
+      <c r="H3" t="str">
+        <f t="shared" ref="H3:H6" si="0">VLOOKUP(G3,A3:E12,2,FALSE)</f>
+        <v>Rohit</v>
+      </c>
+      <c r="I3" t="str">
+        <f t="shared" ref="I3:I6" si="1">VLOOKUP(G3,A3:E12,3,FALSE)</f>
+        <v>Finance</v>
+      </c>
+      <c r="J3">
+        <f t="shared" ref="J3:J6" si="2">VLOOKUP(G3,A3:E12,4,FALSE)</f>
+        <v>55000</v>
+      </c>
+      <c r="K3" t="str">
+        <f t="shared" ref="K3:K6" si="3">VLOOKUP(G3,A3:E12,5,FALSE)</f>
+        <v>Delhi</v>
+      </c>
+      <c r="M3" t="s">
+        <v>180</v>
+      </c>
+      <c r="N3" t="str">
+        <f t="shared" ref="N3:N6" si="4">_xlfn.XLOOKUP(M3,A3:A12,B3:B12)</f>
+        <v>Sneha</v>
+      </c>
+      <c r="O3" t="str">
+        <f t="shared" ref="O3:O6" si="5">_xlfn.XLOOKUP(M3,A3:A12,C3:C12)</f>
+        <v>IT</v>
+      </c>
+      <c r="P3">
+        <f t="shared" ref="P3:P6" si="6">_xlfn.XLOOKUP(M3,A3:A12,D3:D12)</f>
+        <v>48000</v>
+      </c>
+      <c r="Q3" t="str">
+        <f t="shared" ref="Q3:Q6" si="7">_xlfn.XLOOKUP(M3,A3:A12,E3:E12)</f>
+        <v>Hyderabad</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D4" s="3">
+        <v>52000</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" t="s">
+        <v>171</v>
+      </c>
+      <c r="H4" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="I4" t="e">
+        <f t="shared" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="J4" t="e">
+        <f t="shared" si="2"/>
+        <v>#N/A</v>
+      </c>
+      <c r="K4" t="e">
+        <f t="shared" si="3"/>
+        <v>#N/A</v>
+      </c>
+      <c r="M4" t="s">
+        <v>188</v>
+      </c>
+      <c r="N4" t="str">
+        <f t="shared" si="4"/>
+        <v>Meera</v>
+      </c>
+      <c r="O4" t="str">
+        <f t="shared" si="5"/>
+        <v>Sales</v>
+      </c>
+      <c r="P4">
+        <f t="shared" si="6"/>
+        <v>43000</v>
+      </c>
+      <c r="Q4" t="str">
+        <f t="shared" si="7"/>
+        <v>Mumbai</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D5" s="3">
+        <v>48000</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" t="s">
+        <v>190</v>
+      </c>
+      <c r="H5" t="str">
+        <f t="shared" si="0"/>
+        <v>Vikram</v>
+      </c>
+      <c r="I5" t="str">
+        <f t="shared" si="1"/>
+        <v>IT</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="2"/>
+        <v>60000</v>
+      </c>
+      <c r="K5" t="str">
+        <f t="shared" si="3"/>
+        <v>Chennai</v>
+      </c>
+      <c r="M5" t="s">
+        <v>182</v>
+      </c>
+      <c r="N5" t="str">
+        <f t="shared" si="4"/>
+        <v>Kiran</v>
+      </c>
+      <c r="O5" t="str">
+        <f t="shared" si="5"/>
+        <v>Sales</v>
+      </c>
+      <c r="P5">
+        <f t="shared" si="6"/>
+        <v>40000</v>
+      </c>
+      <c r="Q5" t="str">
+        <f t="shared" si="7"/>
+        <v>Bangalore</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="3">
+        <v>40000</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="G6" t="s">
+        <v>184</v>
+      </c>
+      <c r="H6" t="str">
+        <f t="shared" si="0"/>
+        <v>Ananya</v>
+      </c>
+      <c r="I6" t="str">
+        <f t="shared" si="1"/>
+        <v>HR</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="2"/>
+        <v>46000</v>
+      </c>
+      <c r="K6" t="str">
+        <f t="shared" si="3"/>
+        <v>Pune</v>
+      </c>
+      <c r="M6" t="s">
+        <v>192</v>
+      </c>
+      <c r="N6" t="str">
+        <f t="shared" si="4"/>
+        <v>Divya</v>
+      </c>
+      <c r="O6" t="str">
+        <f t="shared" si="5"/>
+        <v>Finance</v>
+      </c>
+      <c r="P6">
+        <f t="shared" si="6"/>
+        <v>51000</v>
+      </c>
+      <c r="Q6" t="str">
+        <f t="shared" si="7"/>
+        <v>Bangalore</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="D7" s="3">
+        <v>46000</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D8" s="3">
+        <v>55000</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" s="3">
+        <v>43000</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A10" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D10" s="3">
+        <v>60000</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D11" s="3">
+        <v>51000</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E1AADFC-86D8-424E-B8C2-CAF7F6746C5B}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>